<commit_message>
Identidad visual LGV Consultora
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantilla_empleados_simulacros.xlsx
+++ b/public/plantilla_empleados_simulacros.xlsx
@@ -119,7 +119,7 @@
     </font>
     <font>
       <b/>
-      <color rgb="FFB91C1C"/>
+      <color rgb="FF1B2A4A"/>
       <sz val="16"/>
       <name val="Arial"/>
     </font>
@@ -157,7 +157,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFB91C1C"/>
+        <fgColor rgb="FF1B2A4A"/>
       </patternFill>
     </fill>
     <fill>
@@ -171,12 +171,21 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFC9A84C"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -200,18 +209,18 @@
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -552,7 +561,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
-    <tabColor rgb="FFB91C1C"/>
+    <tabColor rgb="FFC9A84C"/>
   </sheetPr>
   <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>

</xml_diff>

<commit_message>
Mejoras en carga de empleados
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantilla_empleados_simulacros.xlsx
+++ b/public/plantilla_empleados_simulacros.xlsx
@@ -27,7 +27,7 @@
     <t>2. En la hoja «Empleados», cargá una fila por empleado a partir de la fila 2, sin cambiar los títulos de la fila 1.</t>
   </si>
   <si>
-    <t>3. El celular va como 549 + característica + número, sin 0, sin 15 y sin espacios (ej: 5492614123456).</t>
+    <t>3. El celular va con la característica y el número, con o sin 0 y 15, con o sin espacios o guiones (ej: 261 610-5828, 0261 15 6105828 o 5492616105828). El sistema lo convierte solo al formato internacional.</t>
   </si>
   <si>
     <t>4. El Rol se elige de la lista desplegable: General, Coordinador o Brigadista.</t>
@@ -592,7 +592,7 @@
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
     </row>
-    <row r="4" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -602,7 +602,7 @@
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
     </row>
-    <row r="5" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" ht="52" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>

</xml_diff>